<commit_message>
chore: regenerate public samples for cardinality fix + move dev docs to .dev/
- Regenerate committed sample reports (html/pdf/annotated) so public
  artifacts reflect v2.3.0: revenue no longer flagged as a duplicate-ID
  column, order_status no longer flagged near-constant.
- Move dev-only docs (CLAUDE/HANDOFF/PLAN/DECISIONS/AUDIT/FAILURES) into
  .dev/ so the public root shows only README, CHANGELOG, LICENSE, source,
  samples, tests.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_mixed_types_annotated.xlsx
+++ b/samples/output/sample_mixed_types_annotated.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,10 +31,6 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -45,14 +41,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-        <bgColor rgb="001F3864"/>
+        <fgColor rgb="001f2e7a"/>
+        <bgColor rgb="001f2e7a"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FADBD8"/>
-        <bgColor rgb="00FADBD8"/>
+        <fgColor rgb="00fce8e7"/>
+        <bgColor rgb="00fce8e7"/>
       </patternFill>
     </fill>
   </fills>
@@ -68,10 +64,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -458,7 +453,7 @@
           <t>revenue</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>revenue_mixed</t>
         </is>
@@ -478,7 +473,7 @@
       <c r="B2" t="n">
         <v>17.07</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="2" t="n">
         <v>17.07</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -496,7 +491,7 @@
       <c r="B3" t="n">
         <v>68.39</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>68.39</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -514,7 +509,7 @@
       <c r="B4" t="n">
         <v>585.1900000000001</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>585.1900000000001</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -532,7 +527,7 @@
       <c r="B5" t="n">
         <v>19.06</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="2" t="n">
         <v>19.06</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -550,7 +545,7 @@
       <c r="B6" t="n">
         <v>111.68</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>111.68</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -568,7 +563,7 @@
       <c r="B7" t="n">
         <v>43.4</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="2" t="n">
         <v>43.4</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -586,7 +581,7 @@
       <c r="B8" t="n">
         <v>175.39</v>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -606,7 +601,7 @@
       <c r="B9" t="n">
         <v>82.84999999999999</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="2" t="n">
         <v>82.84999999999999</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -624,7 +619,7 @@
       <c r="B10" t="n">
         <v>1361.16</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="2" t="n">
         <v>1361.16</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -642,7 +637,7 @@
       <c r="B11" t="n">
         <v>317.31</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="2" t="n">
         <v>317.31</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -660,7 +655,7 @@
       <c r="B12" t="n">
         <v>20.74</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="2" t="n">
         <v>20.74</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -678,7 +673,7 @@
       <c r="B13" t="n">
         <v>406.2</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="2" t="n">
         <v>406.2</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -696,7 +691,7 @@
       <c r="B14" t="n">
         <v>46.43</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="2" t="n">
         <v>46.43</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -714,7 +709,7 @@
       <c r="B15" t="n">
         <v>62.46</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="2" t="n">
         <v>62.46</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -732,7 +727,7 @@
       <c r="B16" t="n">
         <v>237.63</v>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="2" t="n">
         <v>237.63</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -750,7 +745,7 @@
       <c r="B17" t="n">
         <v>70.98</v>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="2" t="n">
         <v>70.98</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -768,7 +763,7 @@
       <c r="B18" t="n">
         <v>566.39</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="2" t="n">
         <v>566.39</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -786,7 +781,7 @@
       <c r="B19" t="n">
         <v>46.44</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="2" t="n">
         <v>46.44</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -804,7 +799,7 @@
       <c r="B20" t="n">
         <v>58.65</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="2" t="n">
         <v>58.65</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -822,7 +817,7 @@
       <c r="B21" t="n">
         <v>55.45</v>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C21" s="2" t="n">
         <v>55.45</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -840,7 +835,7 @@
       <c r="B22" t="n">
         <v>63.53</v>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -860,7 +855,7 @@
       <c r="B23" t="n">
         <v>771.85</v>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C23" s="2" t="n">
         <v>771.85</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -878,7 +873,7 @@
       <c r="B24" t="n">
         <v>381.15</v>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C24" s="2" t="n">
         <v>381.15</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -896,7 +891,7 @@
       <c r="B25" t="n">
         <v>1929.31</v>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C25" s="2" t="n">
         <v>1929.31</v>
       </c>
       <c r="D25" t="inlineStr">
@@ -914,7 +909,7 @@
       <c r="B26" t="n">
         <v>4453.59</v>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -934,7 +929,7 @@
       <c r="B27" t="n">
         <v>31.62</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C27" s="2" t="n">
         <v>31.62</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -952,7 +947,7 @@
       <c r="B28" t="n">
         <v>164.95</v>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C28" s="2" t="n">
         <v>164.95</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -970,7 +965,7 @@
       <c r="B29" t="n">
         <v>25.42</v>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C29" s="2" t="n">
         <v>25.42</v>
       </c>
       <c r="D29" t="inlineStr">
@@ -988,7 +983,7 @@
       <c r="B30" t="n">
         <v>46.23</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" s="2" t="n">
         <v>46.23</v>
       </c>
       <c r="D30" t="inlineStr">
@@ -1006,7 +1001,7 @@
       <c r="B31" t="n">
         <v>57.68</v>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1026,7 +1021,7 @@
       <c r="B32" t="n">
         <v>30.39</v>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C32" s="2" t="n">
         <v>30.39</v>
       </c>
       <c r="D32" t="inlineStr">
@@ -1044,7 +1039,7 @@
       <c r="B33" t="n">
         <v>30.64</v>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C33" s="2" t="n">
         <v>30.64</v>
       </c>
       <c r="D33" t="inlineStr">
@@ -1062,7 +1057,7 @@
       <c r="B34" t="n">
         <v>119.53</v>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C34" s="2" t="n">
         <v>119.53</v>
       </c>
       <c r="D34" t="inlineStr">
@@ -1080,7 +1075,7 @@
       <c r="B35" t="n">
         <v>23.92</v>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C35" s="2" t="n">
         <v>23.92</v>
       </c>
       <c r="D35" t="inlineStr">
@@ -1098,7 +1093,7 @@
       <c r="B36" t="n">
         <v>524.89</v>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="C36" s="2" t="n">
         <v>524.89</v>
       </c>
       <c r="D36" t="inlineStr">
@@ -1116,7 +1111,7 @@
       <c r="B37" t="n">
         <v>37.46</v>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C37" s="2" t="n">
         <v>37.46</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -1134,7 +1129,7 @@
       <c r="B38" t="n">
         <v>10040.21</v>
       </c>
-      <c r="C38" s="3" t="n">
+      <c r="C38" s="2" t="n">
         <v>10040.21</v>
       </c>
       <c r="D38" t="inlineStr">
@@ -1152,7 +1147,7 @@
       <c r="B39" t="n">
         <v>75.41</v>
       </c>
-      <c r="C39" s="3" t="n">
+      <c r="C39" s="2" t="n">
         <v>75.41</v>
       </c>
       <c r="D39" t="inlineStr">
@@ -1170,7 +1165,7 @@
       <c r="B40" t="n">
         <v>165.34</v>
       </c>
-      <c r="C40" s="3" t="n">
+      <c r="C40" s="2" t="n">
         <v>165.34</v>
       </c>
       <c r="D40" t="inlineStr">
@@ -1188,7 +1183,7 @@
       <c r="B41" t="n">
         <v>21.26</v>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="C41" s="2" t="n">
         <v>21.26</v>
       </c>
       <c r="D41" t="inlineStr">
@@ -1206,7 +1201,7 @@
       <c r="B42" t="n">
         <v>1918.19</v>
       </c>
-      <c r="C42" s="3" t="n">
+      <c r="C42" s="2" t="n">
         <v>1918.19</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -1224,7 +1219,7 @@
       <c r="B43" t="n">
         <v>795.72</v>
       </c>
-      <c r="C43" s="3" t="n">
+      <c r="C43" s="2" t="n">
         <v>795.72</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -1242,7 +1237,7 @@
       <c r="B44" t="n">
         <v>231.68</v>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="C44" s="2" t="n">
         <v>231.68</v>
       </c>
       <c r="D44" t="inlineStr">
@@ -1260,7 +1255,7 @@
       <c r="B45" t="n">
         <v>19.68</v>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1280,7 +1275,7 @@
       <c r="B46" t="n">
         <v>203.57</v>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="C46" s="2" t="n">
         <v>203.57</v>
       </c>
       <c r="D46" t="inlineStr">
@@ -1298,7 +1293,7 @@
       <c r="B47" t="n">
         <v>27.6</v>
       </c>
-      <c r="C47" s="3" t="n">
+      <c r="C47" s="2" t="n">
         <v>27.6</v>
       </c>
       <c r="D47" t="inlineStr">
@@ -1316,7 +1311,7 @@
       <c r="B48" t="n">
         <v>1330.8</v>
       </c>
-      <c r="C48" s="3" t="n">
+      <c r="C48" s="2" t="n">
         <v>1330.8</v>
       </c>
       <c r="D48" t="inlineStr">
@@ -1334,7 +1329,7 @@
       <c r="B49" t="n">
         <v>499.59</v>
       </c>
-      <c r="C49" s="3" t="n">
+      <c r="C49" s="2" t="n">
         <v>499.59</v>
       </c>
       <c r="D49" t="inlineStr">
@@ -1352,7 +1347,7 @@
       <c r="B50" t="n">
         <v>171.26</v>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="C50" s="2" t="n">
         <v>171.26</v>
       </c>
       <c r="D50" t="inlineStr">
@@ -1370,7 +1365,7 @@
       <c r="B51" t="n">
         <v>3.84</v>
       </c>
-      <c r="C51" s="3" t="n">
+      <c r="C51" s="2" t="n">
         <v>3.84</v>
       </c>
       <c r="D51" t="inlineStr">
@@ -1388,7 +1383,7 @@
       <c r="B52" t="n">
         <v>33.95</v>
       </c>
-      <c r="C52" s="3" t="n">
+      <c r="C52" s="2" t="n">
         <v>33.95</v>
       </c>
       <c r="D52" t="inlineStr">
@@ -1406,7 +1401,7 @@
       <c r="B53" t="n">
         <v>416.4</v>
       </c>
-      <c r="C53" s="3" t="n">
+      <c r="C53" s="2" t="n">
         <v>416.4</v>
       </c>
       <c r="D53" t="inlineStr">
@@ -1424,7 +1419,7 @@
       <c r="B54" t="n">
         <v>915.37</v>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1444,7 +1439,7 @@
       <c r="B55" t="n">
         <v>783.49</v>
       </c>
-      <c r="C55" s="3" t="n">
+      <c r="C55" s="2" t="n">
         <v>783.49</v>
       </c>
       <c r="D55" t="inlineStr">
@@ -1462,7 +1457,7 @@
       <c r="B56" t="n">
         <v>13.63</v>
       </c>
-      <c r="C56" s="3" t="n">
+      <c r="C56" s="2" t="n">
         <v>13.63</v>
       </c>
       <c r="D56" t="inlineStr">
@@ -1480,7 +1475,7 @@
       <c r="B57" t="n">
         <v>233.3</v>
       </c>
-      <c r="C57" s="3" t="n">
+      <c r="C57" s="2" t="n">
         <v>233.3</v>
       </c>
       <c r="D57" t="inlineStr">
@@ -1498,7 +1493,7 @@
       <c r="B58" t="n">
         <v>680.8</v>
       </c>
-      <c r="C58" s="3" t="n">
+      <c r="C58" s="2" t="n">
         <v>680.8</v>
       </c>
       <c r="D58" t="inlineStr">
@@ -1516,7 +1511,7 @@
       <c r="B59" t="n">
         <v>12.34</v>
       </c>
-      <c r="C59" s="3" t="n">
+      <c r="C59" s="2" t="n">
         <v>12.34</v>
       </c>
       <c r="D59" t="inlineStr">
@@ -1534,7 +1529,7 @@
       <c r="B60" t="n">
         <v>146.66</v>
       </c>
-      <c r="C60" s="3" t="n">
+      <c r="C60" s="2" t="n">
         <v>146.66</v>
       </c>
       <c r="D60" t="inlineStr">
@@ -1552,7 +1547,7 @@
       <c r="B61" t="n">
         <v>223.8</v>
       </c>
-      <c r="C61" s="3" t="n">
+      <c r="C61" s="2" t="n">
         <v>223.8</v>
       </c>
       <c r="D61" t="inlineStr">
@@ -1570,7 +1565,7 @@
       <c r="B62" t="n">
         <v>94.52</v>
       </c>
-      <c r="C62" s="3" t="n">
+      <c r="C62" s="2" t="n">
         <v>94.52</v>
       </c>
       <c r="D62" t="inlineStr">
@@ -1588,7 +1583,7 @@
       <c r="B63" t="n">
         <v>9.220000000000001</v>
       </c>
-      <c r="C63" s="3" t="n">
+      <c r="C63" s="2" t="n">
         <v>9.220000000000001</v>
       </c>
       <c r="D63" t="inlineStr">
@@ -1606,7 +1601,7 @@
       <c r="B64" t="n">
         <v>91.05</v>
       </c>
-      <c r="C64" s="3" t="n">
+      <c r="C64" s="2" t="n">
         <v>91.05</v>
       </c>
       <c r="D64" t="inlineStr">
@@ -1624,7 +1619,7 @@
       <c r="B65" t="n">
         <v>90.83</v>
       </c>
-      <c r="C65" s="3" t="n">
+      <c r="C65" s="2" t="n">
         <v>90.83</v>
       </c>
       <c r="D65" t="inlineStr">
@@ -1642,7 +1637,7 @@
       <c r="B66" t="n">
         <v>118.85</v>
       </c>
-      <c r="C66" s="3" t="n">
+      <c r="C66" s="2" t="n">
         <v>118.85</v>
       </c>
       <c r="D66" t="inlineStr">
@@ -1660,7 +1655,7 @@
       <c r="B67" t="n">
         <v>63.74</v>
       </c>
-      <c r="C67" s="3" t="n">
+      <c r="C67" s="2" t="n">
         <v>63.74</v>
       </c>
       <c r="D67" t="inlineStr">
@@ -1678,7 +1673,7 @@
       <c r="B68" t="n">
         <v>76.36</v>
       </c>
-      <c r="C68" s="3" t="n">
+      <c r="C68" s="2" t="n">
         <v>76.36</v>
       </c>
       <c r="D68" t="inlineStr">
@@ -1696,7 +1691,7 @@
       <c r="B69" t="n">
         <v>139.83</v>
       </c>
-      <c r="C69" s="3" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1716,7 +1711,7 @@
       <c r="B70" t="n">
         <v>288.21</v>
       </c>
-      <c r="C70" s="3" t="n">
+      <c r="C70" s="2" t="n">
         <v>288.21</v>
       </c>
       <c r="D70" t="inlineStr">
@@ -1734,7 +1729,7 @@
       <c r="B71" t="n">
         <v>94.01000000000001</v>
       </c>
-      <c r="C71" s="3" t="n">
+      <c r="C71" s="2" t="n">
         <v>94.01000000000001</v>
       </c>
       <c r="D71" t="inlineStr">
@@ -1752,7 +1747,7 @@
       <c r="B72" t="n">
         <v>80.28</v>
       </c>
-      <c r="C72" s="3" t="n">
+      <c r="C72" s="2" t="n">
         <v>80.28</v>
       </c>
       <c r="D72" t="inlineStr">
@@ -1770,7 +1765,7 @@
       <c r="B73" t="n">
         <v>170.47</v>
       </c>
-      <c r="C73" s="3" t="n">
+      <c r="C73" s="2" t="n">
         <v>170.47</v>
       </c>
       <c r="D73" t="inlineStr">
@@ -1788,7 +1783,7 @@
       <c r="B74" t="n">
         <v>8.32</v>
       </c>
-      <c r="C74" s="3" t="n">
+      <c r="C74" s="2" t="n">
         <v>8.32</v>
       </c>
       <c r="D74" t="inlineStr">
@@ -1806,7 +1801,7 @@
       <c r="B75" t="n">
         <v>303.55</v>
       </c>
-      <c r="C75" s="3" t="n">
+      <c r="C75" s="2" t="n">
         <v>303.55</v>
       </c>
       <c r="D75" t="inlineStr">
@@ -1824,7 +1819,7 @@
       <c r="B76" t="n">
         <v>148.29</v>
       </c>
-      <c r="C76" s="3" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1844,7 +1839,7 @@
       <c r="B77" t="n">
         <v>157.52</v>
       </c>
-      <c r="C77" s="3" t="n">
+      <c r="C77" s="2" t="n">
         <v>157.52</v>
       </c>
       <c r="D77" t="inlineStr">
@@ -1862,7 +1857,7 @@
       <c r="B78" t="n">
         <v>627.1</v>
       </c>
-      <c r="C78" s="3" t="n">
+      <c r="C78" s="2" t="n">
         <v>627.1</v>
       </c>
       <c r="D78" t="inlineStr">
@@ -1880,7 +1875,7 @@
       <c r="B79" t="n">
         <v>7.93</v>
       </c>
-      <c r="C79" s="3" t="n">
+      <c r="C79" s="2" t="n">
         <v>7.93</v>
       </c>
       <c r="D79" t="inlineStr">
@@ -1898,7 +1893,7 @@
       <c r="B80" t="n">
         <v>7.68</v>
       </c>
-      <c r="C80" s="3" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1918,7 +1913,7 @@
       <c r="B81" t="n">
         <v>223.79</v>
       </c>
-      <c r="C81" s="3" t="n">
+      <c r="C81" s="2" t="n">
         <v>223.79</v>
       </c>
       <c r="D81" t="inlineStr">
@@ -1936,7 +1931,7 @@
       <c r="B82" t="n">
         <v>146.84</v>
       </c>
-      <c r="C82" s="3" t="n">
+      <c r="C82" s="2" t="n">
         <v>146.84</v>
       </c>
       <c r="D82" t="inlineStr">
@@ -1954,7 +1949,7 @@
       <c r="B83" t="n">
         <v>191.57</v>
       </c>
-      <c r="C83" s="3" t="n">
+      <c r="C83" s="2" t="n">
         <v>191.57</v>
       </c>
       <c r="D83" t="inlineStr">
@@ -1972,7 +1967,7 @@
       <c r="B84" t="n">
         <v>74.2</v>
       </c>
-      <c r="C84" s="3" t="n">
+      <c r="C84" s="2" t="n">
         <v>74.2</v>
       </c>
       <c r="D84" t="inlineStr">
@@ -1990,7 +1985,7 @@
       <c r="B85" t="n">
         <v>402.03</v>
       </c>
-      <c r="C85" s="3" t="n">
+      <c r="C85" s="2" t="n">
         <v>402.03</v>
       </c>
       <c r="D85" t="inlineStr">
@@ -2008,7 +2003,7 @@
       <c r="B86" t="n">
         <v>601.22</v>
       </c>
-      <c r="C86" s="3" t="n">
+      <c r="C86" s="2" t="n">
         <v>601.22</v>
       </c>
       <c r="D86" t="inlineStr">
@@ -2026,7 +2021,7 @@
       <c r="B87" t="n">
         <v>306.73</v>
       </c>
-      <c r="C87" s="3" t="n">
+      <c r="C87" s="2" t="n">
         <v>306.73</v>
       </c>
       <c r="D87" t="inlineStr">
@@ -2044,7 +2039,7 @@
       <c r="B88" t="n">
         <v>100.36</v>
       </c>
-      <c r="C88" s="3" t="n">
+      <c r="C88" s="2" t="n">
         <v>100.36</v>
       </c>
       <c r="D88" t="inlineStr">
@@ -2062,7 +2057,7 @@
       <c r="B89" t="n">
         <v>6.29</v>
       </c>
-      <c r="C89" s="3" t="n">
+      <c r="C89" s="2" t="n">
         <v>6.29</v>
       </c>
       <c r="D89" t="inlineStr">
@@ -2080,7 +2075,7 @@
       <c r="B90" t="n">
         <v>470.53</v>
       </c>
-      <c r="C90" s="3" t="n">
+      <c r="C90" s="2" t="n">
         <v>470.53</v>
       </c>
       <c r="D90" t="inlineStr">
@@ -2098,7 +2093,7 @@
       <c r="B91" t="n">
         <v>927.59</v>
       </c>
-      <c r="C91" s="3" t="n">
+      <c r="C91" s="2" t="n">
         <v>927.59</v>
       </c>
       <c r="D91" t="inlineStr">
@@ -2116,7 +2111,7 @@
       <c r="B92" t="n">
         <v>390.27</v>
       </c>
-      <c r="C92" s="3" t="n">
+      <c r="C92" s="2" t="n">
         <v>390.27</v>
       </c>
       <c r="D92" t="inlineStr">
@@ -2134,7 +2129,7 @@
       <c r="B93" t="n">
         <v>39.67</v>
       </c>
-      <c r="C93" s="3" t="n">
+      <c r="C93" s="2" t="n">
         <v>39.67</v>
       </c>
       <c r="D93" t="inlineStr">
@@ -2152,7 +2147,7 @@
       <c r="B94" t="n">
         <v>407.77</v>
       </c>
-      <c r="C94" s="3" t="n">
+      <c r="C94" s="2" t="n">
         <v>407.77</v>
       </c>
       <c r="D94" t="inlineStr">
@@ -2170,7 +2165,7 @@
       <c r="B95" t="n">
         <v>539.58</v>
       </c>
-      <c r="C95" s="3" t="n">
+      <c r="C95" s="2" t="n">
         <v>539.58</v>
       </c>
       <c r="D95" t="inlineStr">
@@ -2188,7 +2183,7 @@
       <c r="B96" t="n">
         <v>1537.98</v>
       </c>
-      <c r="C96" s="3" t="n">
+      <c r="C96" s="2" t="n">
         <v>1537.98</v>
       </c>
       <c r="D96" t="inlineStr">
@@ -2206,7 +2201,7 @@
       <c r="B97" t="n">
         <v>39.88</v>
       </c>
-      <c r="C97" s="3" t="n">
+      <c r="C97" s="2" t="n">
         <v>39.88</v>
       </c>
       <c r="D97" t="inlineStr">
@@ -2224,7 +2219,7 @@
       <c r="B98" t="n">
         <v>105.67</v>
       </c>
-      <c r="C98" s="3" t="n">
+      <c r="C98" s="2" t="n">
         <v>105.67</v>
       </c>
       <c r="D98" t="inlineStr">
@@ -2242,7 +2237,7 @@
       <c r="B99" t="n">
         <v>455.28</v>
       </c>
-      <c r="C99" s="3" t="n">
+      <c r="C99" s="2" t="n">
         <v>455.28</v>
       </c>
       <c r="D99" t="inlineStr">
@@ -2260,7 +2255,7 @@
       <c r="B100" t="n">
         <v>161.76</v>
       </c>
-      <c r="C100" s="3" t="n">
+      <c r="C100" s="2" t="n">
         <v>161.76</v>
       </c>
       <c r="D100" t="inlineStr">
@@ -2278,7 +2273,7 @@
       <c r="B101" t="n">
         <v>27.77</v>
       </c>
-      <c r="C101" s="3" t="n">
+      <c r="C101" s="2" t="n">
         <v>27.77</v>
       </c>
       <c r="D101" t="inlineStr">
@@ -2296,7 +2291,7 @@
       <c r="B102" t="n">
         <v>276.42</v>
       </c>
-      <c r="C102" s="3" t="n">
+      <c r="C102" s="2" t="n">
         <v>276.42</v>
       </c>
       <c r="D102" t="inlineStr">
@@ -2314,7 +2309,7 @@
       <c r="B103" t="n">
         <v>353.54</v>
       </c>
-      <c r="C103" s="3" t="inlineStr">
+      <c r="C103" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2334,7 +2329,7 @@
       <c r="B104" t="n">
         <v>169.35</v>
       </c>
-      <c r="C104" s="3" t="n">
+      <c r="C104" s="2" t="n">
         <v>169.35</v>
       </c>
       <c r="D104" t="inlineStr">
@@ -2352,7 +2347,7 @@
       <c r="B105" t="n">
         <v>206.31</v>
       </c>
-      <c r="C105" s="3" t="n">
+      <c r="C105" s="2" t="n">
         <v>206.31</v>
       </c>
       <c r="D105" t="inlineStr">
@@ -2370,7 +2365,7 @@
       <c r="B106" t="n">
         <v>100.68</v>
       </c>
-      <c r="C106" s="3" t="n">
+      <c r="C106" s="2" t="n">
         <v>100.68</v>
       </c>
       <c r="D106" t="inlineStr">
@@ -2388,7 +2383,7 @@
       <c r="B107" t="n">
         <v>1362.97</v>
       </c>
-      <c r="C107" s="3" t="n">
+      <c r="C107" s="2" t="n">
         <v>1362.97</v>
       </c>
       <c r="D107" t="inlineStr">
@@ -2406,7 +2401,7 @@
       <c r="B108" t="n">
         <v>38.43</v>
       </c>
-      <c r="C108" s="3" t="n">
+      <c r="C108" s="2" t="n">
         <v>38.43</v>
       </c>
       <c r="D108" t="inlineStr">
@@ -2424,7 +2419,7 @@
       <c r="B109" t="n">
         <v>61.5</v>
       </c>
-      <c r="C109" s="3" t="n">
+      <c r="C109" s="2" t="n">
         <v>61.5</v>
       </c>
       <c r="D109" t="inlineStr">
@@ -2442,7 +2437,7 @@
       <c r="B110" t="n">
         <v>150.88</v>
       </c>
-      <c r="C110" s="3" t="n">
+      <c r="C110" s="2" t="n">
         <v>150.88</v>
       </c>
       <c r="D110" t="inlineStr">
@@ -2460,7 +2455,7 @@
       <c r="B111" t="n">
         <v>554.7</v>
       </c>
-      <c r="C111" s="3" t="n">
+      <c r="C111" s="2" t="n">
         <v>554.7</v>
       </c>
       <c r="D111" t="inlineStr">
@@ -2478,7 +2473,7 @@
       <c r="B112" t="n">
         <v>15.7</v>
       </c>
-      <c r="C112" s="3" t="n">
+      <c r="C112" s="2" t="n">
         <v>15.7</v>
       </c>
       <c r="D112" t="inlineStr">
@@ -2496,7 +2491,7 @@
       <c r="B113" t="n">
         <v>20.79</v>
       </c>
-      <c r="C113" s="3" t="n">
+      <c r="C113" s="2" t="n">
         <v>20.79</v>
       </c>
       <c r="D113" t="inlineStr">
@@ -2514,7 +2509,7 @@
       <c r="B114" t="n">
         <v>6.98</v>
       </c>
-      <c r="C114" s="3" t="n">
+      <c r="C114" s="2" t="n">
         <v>6.98</v>
       </c>
       <c r="D114" t="inlineStr">
@@ -2532,7 +2527,7 @@
       <c r="B115" t="n">
         <v>155.87</v>
       </c>
-      <c r="C115" s="3" t="n">
+      <c r="C115" s="2" t="n">
         <v>155.87</v>
       </c>
       <c r="D115" t="inlineStr">
@@ -2550,7 +2545,7 @@
       <c r="B116" t="n">
         <v>27.73</v>
       </c>
-      <c r="C116" s="3" t="n">
+      <c r="C116" s="2" t="n">
         <v>27.73</v>
       </c>
       <c r="D116" t="inlineStr">
@@ -2568,7 +2563,7 @@
       <c r="B117" t="n">
         <v>83.36</v>
       </c>
-      <c r="C117" s="3" t="n">
+      <c r="C117" s="2" t="n">
         <v>83.36</v>
       </c>
       <c r="D117" t="inlineStr">
@@ -2586,7 +2581,7 @@
       <c r="B118" t="n">
         <v>400.24</v>
       </c>
-      <c r="C118" s="3" t="n">
+      <c r="C118" s="2" t="n">
         <v>400.24</v>
       </c>
       <c r="D118" t="inlineStr">
@@ -2604,7 +2599,7 @@
       <c r="B119" t="n">
         <v>56.69</v>
       </c>
-      <c r="C119" s="3" t="n">
+      <c r="C119" s="2" t="n">
         <v>56.69</v>
       </c>
       <c r="D119" t="inlineStr">
@@ -2622,7 +2617,7 @@
       <c r="B120" t="n">
         <v>209.96</v>
       </c>
-      <c r="C120" s="3" t="n">
+      <c r="C120" s="2" t="n">
         <v>209.96</v>
       </c>
       <c r="D120" t="inlineStr">
@@ -2640,7 +2635,7 @@
       <c r="B121" t="n">
         <v>94.73</v>
       </c>
-      <c r="C121" s="3" t="n">
+      <c r="C121" s="2" t="n">
         <v>94.73</v>
       </c>
       <c r="D121" t="inlineStr">
@@ -2658,7 +2653,7 @@
       <c r="B122" t="n">
         <v>406.74</v>
       </c>
-      <c r="C122" s="3" t="inlineStr">
+      <c r="C122" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2678,7 +2673,7 @@
       <c r="B123" t="n">
         <v>302.68</v>
       </c>
-      <c r="C123" s="3" t="inlineStr">
+      <c r="C123" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2698,7 +2693,7 @@
       <c r="B124" t="n">
         <v>52.57</v>
       </c>
-      <c r="C124" s="3" t="n">
+      <c r="C124" s="2" t="n">
         <v>52.57</v>
       </c>
       <c r="D124" t="inlineStr">
@@ -2716,7 +2711,7 @@
       <c r="B125" t="n">
         <v>115.24</v>
       </c>
-      <c r="C125" s="3" t="n">
+      <c r="C125" s="2" t="n">
         <v>115.24</v>
       </c>
       <c r="D125" t="inlineStr">
@@ -2734,7 +2729,7 @@
       <c r="B126" t="n">
         <v>710.25</v>
       </c>
-      <c r="C126" s="3" t="n">
+      <c r="C126" s="2" t="n">
         <v>710.25</v>
       </c>
       <c r="D126" t="inlineStr">
@@ -2752,7 +2747,7 @@
       <c r="B127" t="n">
         <v>267.75</v>
       </c>
-      <c r="C127" s="3" t="inlineStr">
+      <c r="C127" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -2772,7 +2767,7 @@
       <c r="B128" t="n">
         <v>18.26</v>
       </c>
-      <c r="C128" s="3" t="n">
+      <c r="C128" s="2" t="n">
         <v>18.26</v>
       </c>
       <c r="D128" t="inlineStr">
@@ -2790,7 +2785,7 @@
       <c r="B129" t="n">
         <v>396.8</v>
       </c>
-      <c r="C129" s="3" t="n">
+      <c r="C129" s="2" t="n">
         <v>396.8</v>
       </c>
       <c r="D129" t="inlineStr">
@@ -2808,7 +2803,7 @@
       <c r="B130" t="n">
         <v>29.17</v>
       </c>
-      <c r="C130" s="3" t="n">
+      <c r="C130" s="2" t="n">
         <v>29.17</v>
       </c>
       <c r="D130" t="inlineStr">
@@ -2826,7 +2821,7 @@
       <c r="B131" t="n">
         <v>1234.93</v>
       </c>
-      <c r="C131" s="3" t="n">
+      <c r="C131" s="2" t="n">
         <v>1234.93</v>
       </c>
       <c r="D131" t="inlineStr">
@@ -2844,7 +2839,7 @@
       <c r="B132" t="n">
         <v>689.63</v>
       </c>
-      <c r="C132" s="3" t="n">
+      <c r="C132" s="2" t="n">
         <v>689.63</v>
       </c>
       <c r="D132" t="inlineStr">
@@ -2862,7 +2857,7 @@
       <c r="B133" t="n">
         <v>229.25</v>
       </c>
-      <c r="C133" s="3" t="n">
+      <c r="C133" s="2" t="n">
         <v>229.25</v>
       </c>
       <c r="D133" t="inlineStr">
@@ -2880,7 +2875,7 @@
       <c r="B134" t="n">
         <v>187.89</v>
       </c>
-      <c r="C134" s="3" t="n">
+      <c r="C134" s="2" t="n">
         <v>187.89</v>
       </c>
       <c r="D134" t="inlineStr">
@@ -2898,7 +2893,7 @@
       <c r="B135" t="n">
         <v>108.47</v>
       </c>
-      <c r="C135" s="3" t="n">
+      <c r="C135" s="2" t="n">
         <v>108.47</v>
       </c>
       <c r="D135" t="inlineStr">
@@ -2916,7 +2911,7 @@
       <c r="B136" t="n">
         <v>410.67</v>
       </c>
-      <c r="C136" s="3" t="n">
+      <c r="C136" s="2" t="n">
         <v>410.67</v>
       </c>
       <c r="D136" t="inlineStr">
@@ -2934,7 +2929,7 @@
       <c r="B137" t="n">
         <v>85.09999999999999</v>
       </c>
-      <c r="C137" s="3" t="n">
+      <c r="C137" s="2" t="n">
         <v>85.09999999999999</v>
       </c>
       <c r="D137" t="inlineStr">
@@ -2952,7 +2947,7 @@
       <c r="B138" t="n">
         <v>211.32</v>
       </c>
-      <c r="C138" s="3" t="n">
+      <c r="C138" s="2" t="n">
         <v>211.32</v>
       </c>
       <c r="D138" t="inlineStr">
@@ -2970,7 +2965,7 @@
       <c r="B139" t="n">
         <v>548.89</v>
       </c>
-      <c r="C139" s="3" t="n">
+      <c r="C139" s="2" t="n">
         <v>548.89</v>
       </c>
       <c r="D139" t="inlineStr">
@@ -2988,7 +2983,7 @@
       <c r="B140" t="n">
         <v>63.9</v>
       </c>
-      <c r="C140" s="3" t="n">
+      <c r="C140" s="2" t="n">
         <v>63.9</v>
       </c>
       <c r="D140" t="inlineStr">
@@ -3006,7 +3001,7 @@
       <c r="B141" t="n">
         <v>58.89</v>
       </c>
-      <c r="C141" s="3" t="n">
+      <c r="C141" s="2" t="n">
         <v>58.89</v>
       </c>
       <c r="D141" t="inlineStr">
@@ -3024,7 +3019,7 @@
       <c r="B142" t="n">
         <v>24.74</v>
       </c>
-      <c r="C142" s="3" t="n">
+      <c r="C142" s="2" t="n">
         <v>24.74</v>
       </c>
       <c r="D142" t="inlineStr">
@@ -3042,7 +3037,7 @@
       <c r="B143" t="n">
         <v>30.06</v>
       </c>
-      <c r="C143" s="3" t="n">
+      <c r="C143" s="2" t="n">
         <v>30.06</v>
       </c>
       <c r="D143" t="inlineStr">
@@ -3060,7 +3055,7 @@
       <c r="B144" t="n">
         <v>9.56</v>
       </c>
-      <c r="C144" s="3" t="n">
+      <c r="C144" s="2" t="n">
         <v>9.56</v>
       </c>
       <c r="D144" t="inlineStr">
@@ -3078,7 +3073,7 @@
       <c r="B145" t="n">
         <v>443.52</v>
       </c>
-      <c r="C145" s="3" t="n">
+      <c r="C145" s="2" t="n">
         <v>443.52</v>
       </c>
       <c r="D145" t="inlineStr">
@@ -3096,7 +3091,7 @@
       <c r="B146" t="n">
         <v>2238.08</v>
       </c>
-      <c r="C146" s="3" t="n">
+      <c r="C146" s="2" t="n">
         <v>2238.08</v>
       </c>
       <c r="D146" t="inlineStr">
@@ -3114,7 +3109,7 @@
       <c r="B147" t="n">
         <v>1258.9</v>
       </c>
-      <c r="C147" s="3" t="n">
+      <c r="C147" s="2" t="n">
         <v>1258.9</v>
       </c>
       <c r="D147" t="inlineStr">
@@ -3132,7 +3127,7 @@
       <c r="B148" t="n">
         <v>12.95</v>
       </c>
-      <c r="C148" s="3" t="n">
+      <c r="C148" s="2" t="n">
         <v>12.95</v>
       </c>
       <c r="D148" t="inlineStr">
@@ -3150,7 +3145,7 @@
       <c r="B149" t="n">
         <v>440.22</v>
       </c>
-      <c r="C149" s="3" t="n">
+      <c r="C149" s="2" t="n">
         <v>440.22</v>
       </c>
       <c r="D149" t="inlineStr">
@@ -3168,7 +3163,7 @@
       <c r="B150" t="n">
         <v>1252.83</v>
       </c>
-      <c r="C150" s="3" t="n">
+      <c r="C150" s="2" t="n">
         <v>1252.83</v>
       </c>
       <c r="D150" t="inlineStr">
@@ -3186,7 +3181,7 @@
       <c r="B151" t="n">
         <v>74.8</v>
       </c>
-      <c r="C151" s="3" t="n">
+      <c r="C151" s="2" t="n">
         <v>74.8</v>
       </c>
       <c r="D151" t="inlineStr">
@@ -3204,7 +3199,7 @@
       <c r="B152" t="n">
         <v>172.81</v>
       </c>
-      <c r="C152" s="3" t="n">
+      <c r="C152" s="2" t="n">
         <v>172.81</v>
       </c>
       <c r="D152" t="inlineStr">
@@ -3222,7 +3217,7 @@
       <c r="B153" t="n">
         <v>7.3</v>
       </c>
-      <c r="C153" s="3" t="n">
+      <c r="C153" s="2" t="n">
         <v>7.3</v>
       </c>
       <c r="D153" t="inlineStr">
@@ -3240,7 +3235,7 @@
       <c r="B154" t="n">
         <v>221.43</v>
       </c>
-      <c r="C154" s="3" t="n">
+      <c r="C154" s="2" t="n">
         <v>221.43</v>
       </c>
       <c r="D154" t="inlineStr">
@@ -3258,7 +3253,7 @@
       <c r="B155" t="n">
         <v>30.1</v>
       </c>
-      <c r="C155" s="3" t="n">
+      <c r="C155" s="2" t="n">
         <v>30.1</v>
       </c>
       <c r="D155" t="inlineStr">
@@ -3276,7 +3271,7 @@
       <c r="B156" t="n">
         <v>200.23</v>
       </c>
-      <c r="C156" s="3" t="n">
+      <c r="C156" s="2" t="n">
         <v>200.23</v>
       </c>
       <c r="D156" t="inlineStr">
@@ -3294,7 +3289,7 @@
       <c r="B157" t="n">
         <v>14.27</v>
       </c>
-      <c r="C157" s="3" t="n">
+      <c r="C157" s="2" t="n">
         <v>14.27</v>
       </c>
       <c r="D157" t="inlineStr">
@@ -3312,7 +3307,7 @@
       <c r="B158" t="n">
         <v>335.05</v>
       </c>
-      <c r="C158" s="3" t="n">
+      <c r="C158" s="2" t="n">
         <v>335.05</v>
       </c>
       <c r="D158" t="inlineStr">
@@ -3330,7 +3325,7 @@
       <c r="B159" t="n">
         <v>690.05</v>
       </c>
-      <c r="C159" s="3" t="n">
+      <c r="C159" s="2" t="n">
         <v>690.05</v>
       </c>
       <c r="D159" t="inlineStr">
@@ -3348,7 +3343,7 @@
       <c r="B160" t="n">
         <v>45.84</v>
       </c>
-      <c r="C160" s="3" t="n">
+      <c r="C160" s="2" t="n">
         <v>45.84</v>
       </c>
       <c r="D160" t="inlineStr">
@@ -3366,7 +3361,7 @@
       <c r="B161" t="n">
         <v>26.97</v>
       </c>
-      <c r="C161" s="3" t="n">
+      <c r="C161" s="2" t="n">
         <v>26.97</v>
       </c>
       <c r="D161" t="inlineStr">
@@ -3384,7 +3379,7 @@
       <c r="B162" t="n">
         <v>5.85</v>
       </c>
-      <c r="C162" s="3" t="n">
+      <c r="C162" s="2" t="n">
         <v>5.85</v>
       </c>
       <c r="D162" t="inlineStr">
@@ -3402,7 +3397,7 @@
       <c r="B163" t="n">
         <v>99.52</v>
       </c>
-      <c r="C163" s="3" t="n">
+      <c r="C163" s="2" t="n">
         <v>99.52</v>
       </c>
       <c r="D163" t="inlineStr">
@@ -3420,7 +3415,7 @@
       <c r="B164" t="n">
         <v>62.03</v>
       </c>
-      <c r="C164" s="3" t="n">
+      <c r="C164" s="2" t="n">
         <v>62.03</v>
       </c>
       <c r="D164" t="inlineStr">
@@ -3438,7 +3433,7 @@
       <c r="B165" t="n">
         <v>14.49</v>
       </c>
-      <c r="C165" s="3" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -3458,7 +3453,7 @@
       <c r="B166" t="n">
         <v>292.81</v>
       </c>
-      <c r="C166" s="3" t="n">
+      <c r="C166" s="2" t="n">
         <v>292.81</v>
       </c>
       <c r="D166" t="inlineStr">
@@ -3476,7 +3471,7 @@
       <c r="B167" t="n">
         <v>75.56999999999999</v>
       </c>
-      <c r="C167" s="3" t="n">
+      <c r="C167" s="2" t="n">
         <v>75.56999999999999</v>
       </c>
       <c r="D167" t="inlineStr">
@@ -3494,7 +3489,7 @@
       <c r="B168" t="n">
         <v>29.56</v>
       </c>
-      <c r="C168" s="3" t="n">
+      <c r="C168" s="2" t="n">
         <v>29.56</v>
       </c>
       <c r="D168" t="inlineStr">
@@ -3512,7 +3507,7 @@
       <c r="B169" t="n">
         <v>64.59999999999999</v>
       </c>
-      <c r="C169" s="3" t="n">
+      <c r="C169" s="2" t="n">
         <v>64.59999999999999</v>
       </c>
       <c r="D169" t="inlineStr">
@@ -3530,7 +3525,7 @@
       <c r="B170" t="n">
         <v>740.23</v>
       </c>
-      <c r="C170" s="3" t="n">
+      <c r="C170" s="2" t="n">
         <v>740.23</v>
       </c>
       <c r="D170" t="inlineStr">
@@ -3548,7 +3543,7 @@
       <c r="B171" t="n">
         <v>366.65</v>
       </c>
-      <c r="C171" s="3" t="inlineStr">
+      <c r="C171" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -3568,7 +3563,7 @@
       <c r="B172" t="n">
         <v>122.11</v>
       </c>
-      <c r="C172" s="3" t="n">
+      <c r="C172" s="2" t="n">
         <v>122.11</v>
       </c>
       <c r="D172" t="inlineStr">
@@ -3586,7 +3581,7 @@
       <c r="B173" t="n">
         <v>375.65</v>
       </c>
-      <c r="C173" s="3" t="n">
+      <c r="C173" s="2" t="n">
         <v>375.65</v>
       </c>
       <c r="D173" t="inlineStr">
@@ -3604,7 +3599,7 @@
       <c r="B174" t="n">
         <v>26.01</v>
       </c>
-      <c r="C174" s="3" t="n">
+      <c r="C174" s="2" t="n">
         <v>26.01</v>
       </c>
       <c r="D174" t="inlineStr">
@@ -3622,7 +3617,7 @@
       <c r="B175" t="n">
         <v>155.8</v>
       </c>
-      <c r="C175" s="3" t="n">
+      <c r="C175" s="2" t="n">
         <v>155.8</v>
       </c>
       <c r="D175" t="inlineStr">
@@ -3640,7 +3635,7 @@
       <c r="B176" t="n">
         <v>185.12</v>
       </c>
-      <c r="C176" s="3" t="n">
+      <c r="C176" s="2" t="n">
         <v>185.12</v>
       </c>
       <c r="D176" t="inlineStr">
@@ -3658,7 +3653,7 @@
       <c r="B177" t="n">
         <v>73.34999999999999</v>
       </c>
-      <c r="C177" s="3" t="n">
+      <c r="C177" s="2" t="n">
         <v>73.34999999999999</v>
       </c>
       <c r="D177" t="inlineStr">
@@ -3676,7 +3671,7 @@
       <c r="B178" t="n">
         <v>285.2</v>
       </c>
-      <c r="C178" s="3" t="n">
+      <c r="C178" s="2" t="n">
         <v>285.2</v>
       </c>
       <c r="D178" t="inlineStr">
@@ -3694,7 +3689,7 @@
       <c r="B179" t="n">
         <v>46.03</v>
       </c>
-      <c r="C179" s="3" t="n">
+      <c r="C179" s="2" t="n">
         <v>46.03</v>
       </c>
       <c r="D179" t="inlineStr">
@@ -3712,7 +3707,7 @@
       <c r="B180" t="n">
         <v>318.85</v>
       </c>
-      <c r="C180" s="3" t="n">
+      <c r="C180" s="2" t="n">
         <v>318.85</v>
       </c>
       <c r="D180" t="inlineStr">
@@ -3730,7 +3725,7 @@
       <c r="B181" t="n">
         <v>339.61</v>
       </c>
-      <c r="C181" s="3" t="n">
+      <c r="C181" s="2" t="n">
         <v>339.61</v>
       </c>
       <c r="D181" t="inlineStr">
@@ -3748,7 +3743,7 @@
       <c r="B182" t="n">
         <v>1.87</v>
       </c>
-      <c r="C182" s="3" t="n">
+      <c r="C182" s="2" t="n">
         <v>1.87</v>
       </c>
       <c r="D182" t="inlineStr">
@@ -3766,7 +3761,7 @@
       <c r="B183" t="n">
         <v>884.89</v>
       </c>
-      <c r="C183" s="3" t="n">
+      <c r="C183" s="2" t="n">
         <v>884.89</v>
       </c>
       <c r="D183" t="inlineStr">
@@ -3784,7 +3779,7 @@
       <c r="B184" t="n">
         <v>1.54</v>
       </c>
-      <c r="C184" s="3" t="n">
+      <c r="C184" s="2" t="n">
         <v>1.54</v>
       </c>
       <c r="D184" t="inlineStr">
@@ -3802,7 +3797,7 @@
       <c r="B185" t="n">
         <v>58.91</v>
       </c>
-      <c r="C185" s="3" t="n">
+      <c r="C185" s="2" t="n">
         <v>58.91</v>
       </c>
       <c r="D185" t="inlineStr">
@@ -3820,7 +3815,7 @@
       <c r="B186" t="n">
         <v>690.92</v>
       </c>
-      <c r="C186" s="3" t="n">
+      <c r="C186" s="2" t="n">
         <v>690.92</v>
       </c>
       <c r="D186" t="inlineStr">
@@ -3838,7 +3833,7 @@
       <c r="B187" t="n">
         <v>92.20999999999999</v>
       </c>
-      <c r="C187" s="3" t="n">
+      <c r="C187" s="2" t="n">
         <v>92.20999999999999</v>
       </c>
       <c r="D187" t="inlineStr">
@@ -3856,7 +3851,7 @@
       <c r="B188" t="n">
         <v>16.46</v>
       </c>
-      <c r="C188" s="3" t="n">
+      <c r="C188" s="2" t="n">
         <v>16.46</v>
       </c>
       <c r="D188" t="inlineStr">
@@ -3874,7 +3869,7 @@
       <c r="B189" t="n">
         <v>28.77</v>
       </c>
-      <c r="C189" s="3" t="n">
+      <c r="C189" s="2" t="n">
         <v>28.77</v>
       </c>
       <c r="D189" t="inlineStr">
@@ -3892,7 +3887,7 @@
       <c r="B190" t="n">
         <v>692.53</v>
       </c>
-      <c r="C190" s="3" t="n">
+      <c r="C190" s="2" t="n">
         <v>692.53</v>
       </c>
       <c r="D190" t="inlineStr">
@@ -3910,7 +3905,7 @@
       <c r="B191" t="n">
         <v>8.31</v>
       </c>
-      <c r="C191" s="3" t="n">
+      <c r="C191" s="2" t="n">
         <v>8.31</v>
       </c>
       <c r="D191" t="inlineStr">
@@ -3928,7 +3923,7 @@
       <c r="B192" t="n">
         <v>807.13</v>
       </c>
-      <c r="C192" s="3" t="n">
+      <c r="C192" s="2" t="n">
         <v>807.13</v>
       </c>
       <c r="D192" t="inlineStr">
@@ -3946,7 +3941,7 @@
       <c r="B193" t="n">
         <v>136.64</v>
       </c>
-      <c r="C193" s="3" t="n">
+      <c r="C193" s="2" t="n">
         <v>136.64</v>
       </c>
       <c r="D193" t="inlineStr">
@@ -3964,7 +3959,7 @@
       <c r="B194" t="n">
         <v>24.81</v>
       </c>
-      <c r="C194" s="3" t="n">
+      <c r="C194" s="2" t="n">
         <v>24.81</v>
       </c>
       <c r="D194" t="inlineStr">
@@ -3982,7 +3977,7 @@
       <c r="B195" t="n">
         <v>61.89</v>
       </c>
-      <c r="C195" s="3" t="n">
+      <c r="C195" s="2" t="n">
         <v>61.89</v>
       </c>
       <c r="D195" t="inlineStr">
@@ -4000,7 +3995,7 @@
       <c r="B196" t="n">
         <v>32.27</v>
       </c>
-      <c r="C196" s="3" t="n">
+      <c r="C196" s="2" t="n">
         <v>32.27</v>
       </c>
       <c r="D196" t="inlineStr">
@@ -4018,7 +4013,7 @@
       <c r="B197" t="n">
         <v>544.21</v>
       </c>
-      <c r="C197" s="3" t="n">
+      <c r="C197" s="2" t="n">
         <v>544.21</v>
       </c>
       <c r="D197" t="inlineStr">
@@ -4036,7 +4031,7 @@
       <c r="B198" t="n">
         <v>445.25</v>
       </c>
-      <c r="C198" s="3" t="n">
+      <c r="C198" s="2" t="n">
         <v>445.25</v>
       </c>
       <c r="D198" t="inlineStr">
@@ -4054,7 +4049,7 @@
       <c r="B199" t="n">
         <v>11.26</v>
       </c>
-      <c r="C199" s="3" t="n">
+      <c r="C199" s="2" t="n">
         <v>11.26</v>
       </c>
       <c r="D199" t="inlineStr">
@@ -4072,7 +4067,7 @@
       <c r="B200" t="n">
         <v>81.01000000000001</v>
       </c>
-      <c r="C200" s="3" t="n">
+      <c r="C200" s="2" t="n">
         <v>81.01000000000001</v>
       </c>
       <c r="D200" t="inlineStr">
@@ -4090,7 +4085,7 @@
       <c r="B201" t="n">
         <v>40.66</v>
       </c>
-      <c r="C201" s="3" t="n">
+      <c r="C201" s="2" t="n">
         <v>40.66</v>
       </c>
       <c r="D201" t="inlineStr">
@@ -4154,64 +4149,64 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>revenue_mixed</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Type Inconsistency</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Column 'revenue_mixed' appears to be purely numeric.</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>However, 15 str values were found among 200 non-null values (the majority type covers 92.5%). Examples of unexpected values: 'N/A', 'N/A', 'N/A', and 2 more.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Review the non-numeric values in 'revenue_mixed' and decide whether they should be converted to numeric, replaced with a proper null, or moved to a separate column.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>revenue_mixed</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Sentinel Value</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Column 'revenue_mixed' appears to be a clean numeric column.</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>However, 7.5% of values (1 distinct sentinel string) are placeholder text rather than real data: 'N/A' (15 times).</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Replace sentinel values in 'revenue_mixed' with proper null/blank cells so that downstream tools handle missing data correctly and row counts reflect reality.</t>
         </is>

</xml_diff>

<commit_message>
Fix favicon palette, add responsive/print CSS, regenerate samples
- Favicon SVG: #1F3864 → #1f2e7a (Chicago-20)
- Add @media (max-width: 640px) responsive breakpoint
- Add @media print styles
- Wrap field inventory table for horizontal scroll on mobile
- Regenerate all sample outputs with current Lailara palette

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_mixed_types_annotated.xlsx
+++ b/samples/output/sample_mixed_types_annotated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Findings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
fix: regenerate PDF and annotated-Excel samples stale since v2.3.3
Companion to the HTML sample refresh. The v2.3.3 health-narrative wording
change lives in the shared _palette.health_assessment_text, which also feeds
the PDF, so the committed PDF/Excel portfolio artifacts carried the old copy.
Regenerated all three from current code (sales PDF verified to contain the
new wording). Not covered by the fidelity test — PDFs embed nondeterministic
metadata and the workbook is binary — so refreshed by hand.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_mixed_types_annotated.xlsx
+++ b/samples/output/sample_mixed_types_annotated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Findings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Align README example output to shipped sample; regenerate samples at v2.4.0
The README "Example Output" block was stale: it claimed 200 rows x 6 columns
and 4 findings (2 Critical / 1 Warning / 1 Info) with a nonexistent `status`
finding. The shipped sample_mixed_types.xlsx is 200 x 4 and the current CLI
reports 2 findings, both Critical on revenue_mixed. Updated the block to the
verbatim current run.

Also regenerated the committed sample artifacts (HTML/PDF for both samples,
annotated Excel for mixed_types) which were still emitted at v2.3.2 — refreshed
to v2.4.0 (version string, print-CSS palette tokens, sales health-assessment
copy). Finding counts unchanged (mixed 2, sales 5). Docs/artifacts only; no
engine or version changes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/output/sample_mixed_types_annotated.xlsx
+++ b/samples/output/sample_mixed_types_annotated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Findings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>